<commit_message>
Refine matching-area hint glow and six-percent pulse
</commit_message>
<xml_diff>
--- a/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
+++ b/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="Reb2cf8d7c7da4da9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="Rc8b5d613959c4da8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -255,7 +255,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -266,7 +266,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -276,7 +276,7 @@
         <x:color rgb="FF475569"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF1F5F9"/>
         </x:patternFill>
       </x:fill>
@@ -286,7 +286,7 @@
         <x:color rgb="FF6D28D9"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEDE9FE"/>
         </x:patternFill>
       </x:fill>
@@ -297,7 +297,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -585,14 +585,14 @@
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Fixed")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
         <x:v>Open / pending</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Open")+COUNTIF(F9:F19,"In progress")</x:f>
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
         <x:v>Clarified</x:v>
@@ -700,7 +700,7 @@
         <x:v>Consolidated into feedback #1; no separate game change.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="58" customHeight="1">
+    <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="28" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -711,17 +711,19 @@
         <x:v>The hint marks around possible gems, while the gem movement is too subtle.</x:v>
       </x:c>
       <x:c r="D11" s="27" t="str">
-        <x:v>Remove the surrounding marks. Move the suggested gems farther and brighten them slightly during the movement.</x:v>
+        <x:v>Keep the marking line. Every gem in the matching area has a slightly brighter glow and a 1.0x–1.06x pulse. Only the two swap gems move inward. Delay and loop smoothly, without overlaps or changes to cells or hit areas.</x:v>
       </x:c>
       <x:c r="E11" s="26" t="str">
         <x:v>Hint / UX</x:v>
       </x:c>
       <x:c r="F11" s="28" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="G11" s="28" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G11" s="28" t="str">
+        <x:v>✓</x:v>
+      </x:c>
       <x:c r="H11" s="27" t="str">
-        <x:v>Handle separately after item 1.</x:v>
+        <x:v>Verified in Unity on 7 Oct 2026 across five gem designs. All-area glow, 6% pulse, no overlaps, touch cancellation and unchanged hit areas passed. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -937,7 +939,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5cc8ded0ccd400f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd415e97d3dd64dd9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add detailed QA fixing report to the Excel tracker
</commit_message>
<xml_diff>
--- a/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
+++ b/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="Rc8b5d613959c4da8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R9648dea607ec4963"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="Rd5d289435ac14867"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,7 +59,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -88,6 +89,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFEF2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -142,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -244,11 +255,50 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="5">
+  <x:dxfs count="7">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -302,6 +352,27 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF6D28D9"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEDE9FE"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -318,6 +389,19 @@
     <x:tableColumn id="6" name="Status"/>
     <x:tableColumn id="7" name="Fixed"/>
     <x:tableColumn id="8" name="Verification / notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FixingReport" displayName="FixingReport" ref="A8:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Feedback"/>
+    <x:tableColumn id="2" name="Change"/>
+    <x:tableColumn id="3" name="Completed work"/>
+    <x:tableColumn id="4" name="Verification / evidence"/>
+    <x:tableColumn id="5" name="Tracker status"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -673,7 +757,7 @@
         <x:v>✓</x:v>
       </x:c>
       <x:c r="H9" s="33" t="str">
-        <x:v>Fixed and visually reviewed on 7 Oct 2026. Local commit 69e0d80.</x:v>
+        <x:v>Fixed and visually reviewed on 7 Oct 2026. Commit 69e0d80d. See Fixing Report for details. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="58" customHeight="1">
@@ -723,7 +807,7 @@
         <x:v>✓</x:v>
       </x:c>
       <x:c r="H11" s="27" t="str">
-        <x:v>Verified in Unity on 7 Oct 2026 across five gem designs. All-area glow, 6% pulse, no overlaps, touch cancellation and unchanged hit areas passed. Phone QA pending.</x:v>
+        <x:v>141 Unity checks passed, 0 failed, on 7 Oct 2026. Commit f6398f84. See Fixing Report for details. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="58" customHeight="1">
@@ -939,7 +1023,453 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd415e97d3dd64dd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22236f5d483a4057"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1D4ED8"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="26"/>
+      <x:c r="B1" s="26"/>
+      <x:c r="C1" s="26"/>
+      <x:c r="D1" s="26"/>
+      <x:c r="E1" s="26"/>
+    </x:row>
+    <x:row r="2" ht="27" customHeight="1">
+      <x:c r="A2" s="43" t="str">
+        <x:v>Royal Throne Fixing Report</x:v>
+      </x:c>
+      <x:c r="B2" s="43"/>
+      <x:c r="C2" s="43"/>
+      <x:c r="D2" s="43"/>
+      <x:c r="E2" s="43"/>
+    </x:row>
+    <x:row r="3" ht="23" customHeight="1">
+      <x:c r="A3" s="45" t="str">
+        <x:v>Updated 7 October 2026. Fixed means implemented and verified in Unity. Physical-phone QA remains pending.</x:v>
+      </x:c>
+      <x:c r="B3" s="45"/>
+      <x:c r="C3" s="45"/>
+      <x:c r="D3" s="45"/>
+      <x:c r="E3" s="45"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="26"/>
+      <x:c r="B4" s="26"/>
+      <x:c r="C4" s="26"/>
+      <x:c r="D4" s="26"/>
+      <x:c r="E4" s="26"/>
+    </x:row>
+    <x:row r="5" ht="25" customHeight="1">
+      <x:c r="A5" s="47" t="str">
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="B5" s="55" t="n">
+        <x:f>'QA Feedback'!D5</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" s="47" t="str">
+        <x:v>Open / pending</x:v>
+      </x:c>
+      <x:c r="D5" s="55" t="n">
+        <x:f>'QA Feedback'!F5</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E5" s="26"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="26"/>
+      <x:c r="B6" s="26"/>
+      <x:c r="C6" s="26"/>
+      <x:c r="D6" s="26"/>
+      <x:c r="E6" s="26"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="26"/>
+      <x:c r="B7" s="26"/>
+      <x:c r="C7" s="26"/>
+      <x:c r="D7" s="26"/>
+      <x:c r="E7" s="26"/>
+    </x:row>
+    <x:row r="8" ht="27" customHeight="1">
+      <x:c r="A8" s="54" t="str">
+        <x:v>Feedback</x:v>
+      </x:c>
+      <x:c r="B8" s="54" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="C8" s="54" t="str">
+        <x:v>Completed work</x:v>
+      </x:c>
+      <x:c r="D8" s="54" t="str">
+        <x:v>Verification / evidence</x:v>
+      </x:c>
+      <x:c r="E8" s="54" t="str">
+        <x:v>Tracker status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="60" customHeight="1">
+      <x:c r="A9" s="48" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B9" s="27" t="str">
+        <x:v>Lives number alignment</x:v>
+      </x:c>
+      <x:c r="C9" s="27" t="str">
+        <x:v>Centered the visible lives number inside the Home heart, following the supplied visual reference.</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="str">
+        <x:v>Reviewed the actual 720 × 1280 Unity homepage and before/after captures. Source compilation passed.</x:v>
+      </x:c>
+      <x:c r="E9" s="48" t="str">
+        <x:f>'QA Feedback'!F9</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" customHeight="1">
+      <x:c r="A10" s="48" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B10" s="27" t="str">
+        <x:v>Duplicate clarification</x:v>
+      </x:c>
+      <x:c r="C10" s="27" t="str">
+        <x:v>The repeated lives-number feedback is tracked under #1. No separate implementation is counted.</x:v>
+      </x:c>
+      <x:c r="D10" s="27" t="str">
+        <x:v>Original QA numbering remains intact in the tracker.</x:v>
+      </x:c>
+      <x:c r="E10" s="48" t="str">
+        <x:f>'QA Feedback'!F10</x:f>
+        <x:v>Clarified</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="60" customHeight="1">
+      <x:c r="A11" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B11" s="27" t="str">
+        <x:v>All-area size pulse</x:v>
+      </x:c>
+      <x:c r="C11" s="27" t="str">
+        <x:v>Every gem inside the matching area, plus both swap partners, grows smoothly from 1.0× to 1.06× and returns.</x:v>
+      </x:c>
+      <x:c r="D11" s="27" t="str">
+        <x:v>Checked six match shapes across five gem designs. Unrelated gems keep their normal size.</x:v>
+      </x:c>
+      <x:c r="E11" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="60" customHeight="1">
+      <x:c r="A12" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B12" s="27" t="str">
+        <x:v>Slightly brighter glow</x:v>
+      </x:c>
+      <x:c r="C12" s="27" t="str">
+        <x:v>All affected gems brighten with the movement. Peak additive brightness is approximately 23%, increased from 16%.</x:v>
+      </x:c>
+      <x:c r="D12" s="27" t="str">
+        <x:v>Confirmed matching sprite overlays, synchronized glow and complete removal on cancellation.</x:v>
+      </x:c>
+      <x:c r="E12" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="60" customHeight="1">
+      <x:c r="A13" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B13" s="27" t="str">
+        <x:v>Two-gem movement</x:v>
+      </x:c>
+      <x:c r="C13" s="27" t="str">
+        <x:v>Only the two swap partners move inward. Their equal travel is limited by the available space between expanded artwork.</x:v>
+      </x:c>
+      <x:c r="D13" s="27" t="str">
+        <x:v>Horizontal and vertical swaps tested. No artwork overlap during either complete sampled loop.</x:v>
+      </x:c>
+      <x:c r="E13" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="60" customHeight="1">
+      <x:c r="A14" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B14" s="27" t="str">
+        <x:v>Gentle start and repeat</x:v>
+      </x:c>
+      <x:c r="C14" s="27" t="str">
+        <x:v>After the existing 1-second idle threshold, wait 0.4 seconds. Approach and return over 1.2 seconds, rest for 0.35 seconds, then repeat.</x:v>
+      </x:c>
+      <x:c r="D14" s="27" t="str">
+        <x:v>Natural idle discovery, the initial pause, two approaches and the return/rest phase passed.</x:v>
+      </x:c>
+      <x:c r="E14" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="60" customHeight="1">
+      <x:c r="A15" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B15" s="27" t="str">
+        <x:v>Marking line retained</x:v>
+      </x:c>
+      <x:c r="C15" s="27" t="str">
+        <x:v>Kept the existing marking line, flowing lights and sparkles around the predicted matching area.</x:v>
+      </x:c>
+      <x:c r="D15" s="27" t="str">
+        <x:v>The line remains visible and follows the full predicted match boundary.</x:v>
+      </x:c>
+      <x:c r="E15" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="60" customHeight="1">
+      <x:c r="A16" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B16" s="27" t="str">
+        <x:v>Cell and input safety</x:v>
+      </x:c>
+      <x:c r="C16" s="27" t="str">
+        <x:v>Animation affects child artwork only. Real cell ownership, gem roots and hit areas remain unchanged.</x:v>
+      </x:c>
+      <x:c r="D16" s="27" t="str">
+        <x:v>Checked roots, colliders and cell ownership throughout live frames. No moves, score, coins or lives were consumed.</x:v>
+      </x:c>
+      <x:c r="E16" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="60" customHeight="1">
+      <x:c r="A17" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B17" s="27" t="str">
+        <x:v>Cancellation and preferences</x:v>
+      </x:c>
+      <x:c r="C17" s="27" t="str">
+        <x:v>Touch, pause, changed gems and invalid hints restore the artwork. Hints OFF clears it. Reduced motion keeps a static readable line.</x:v>
+      </x:c>
+      <x:c r="D17" s="27" t="str">
+        <x:v>Input callbacks, invalidation, pause, destroyed gems, hint settings and reduced-motion checks passed.</x:v>
+      </x:c>
+      <x:c r="E17" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="60" customHeight="1">
+      <x:c r="A18" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B18" s="27" t="str">
+        <x:v>Final verification</x:v>
+      </x:c>
+      <x:c r="C18" s="27" t="str">
+        <x:v>Unity 6000.5.10f1 compiled the change. The focused suite completed with 141 checks passed and 0 failed.</x:v>
+      </x:c>
+      <x:c r="D18" s="27" t="str">
+        <x:v>No runtime errors reported. Reviewed native 720 × 1280 captures and a 3.66-second animation preview.</x:v>
+      </x:c>
+      <x:c r="E18" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="60" customHeight="1">
+      <x:c r="A19" s="48" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B19" s="27" t="str">
+        <x:v>Player profile restored</x:v>
+      </x:c>
+      <x:c r="C19" s="27" t="str">
+        <x:v>Used an isolated QA profile and disposable test board, then restored normal player state.</x:v>
+      </x:c>
+      <x:c r="D19" s="27" t="str">
+        <x:v>Confirmed restored balance and lives, disabled QA routing, no active test runner and a clean scene.</x:v>
+      </x:c>
+      <x:c r="E19" s="48" t="str">
+        <x:f>'QA Feedback'!F11</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="26"/>
+      <x:c r="B20" s="26"/>
+      <x:c r="C20" s="26"/>
+      <x:c r="D20" s="26"/>
+      <x:c r="E20" s="26"/>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21" s="49" t="str">
+        <x:v>Remaining QA and open feedback</x:v>
+      </x:c>
+      <x:c r="B21" s="49"/>
+      <x:c r="C21" s="49"/>
+      <x:c r="D21" s="49"/>
+      <x:c r="E21" s="49"/>
+    </x:row>
+    <x:row r="22" ht="27" customHeight="1">
+      <x:c r="A22" s="54" t="str">
+        <x:v>Feedback</x:v>
+      </x:c>
+      <x:c r="B22" s="54" t="str">
+        <x:v>Follow-up</x:v>
+      </x:c>
+      <x:c r="C22" s="54" t="str">
+        <x:v>Current scope</x:v>
+      </x:c>
+      <x:c r="D22" s="54" t="str">
+        <x:v>Verification needed</x:v>
+      </x:c>
+      <x:c r="E22" s="54" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="60" customHeight="1">
+      <x:c r="A23" s="48" t="str">
+        <x:v>1, 3</x:v>
+      </x:c>
+      <x:c r="B23" s="27" t="str">
+        <x:v>Android and phone QA</x:v>
+      </x:c>
+      <x:c r="C23" s="27" t="str">
+        <x:v>Desktop Unity verification is complete. No updated Android build or physical-phone run was performed.</x:v>
+      </x:c>
+      <x:c r="D23" s="27" t="str">
+        <x:v>Build the updated QA APK and review alignment, motion, glow and touch behaviour on physical phones.</x:v>
+      </x:c>
+      <x:c r="E23" s="27" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="60" customHeight="1">
+      <x:c r="A24" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B24" s="27" t="str">
+        <x:v>Hint accuracy</x:v>
+      </x:c>
+      <x:c r="C24" s="27" t="str">
+        <x:v>The concern about the line indicating multiple moves remains a separate open QA item.</x:v>
+      </x:c>
+      <x:c r="D24" s="27" t="str">
+        <x:v>Investigate hint selection and the marked result before changing this behaviour.</x:v>
+      </x:c>
+      <x:c r="E24" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="60" customHeight="1">
+      <x:c r="A25" s="48" t="str">
+        <x:v>5–11</x:v>
+      </x:c>
+      <x:c r="B25" s="27" t="str">
+        <x:v>Other original QA items</x:v>
+      </x:c>
+      <x:c r="C25" s="27" t="str">
+        <x:v>Fuse fire, special-piece creation, match timing, stuck gems, Color Ball duration and the 2×2-plus-one rule remain open.</x:v>
+      </x:c>
+      <x:c r="D25" s="27" t="str">
+        <x:v>Continue one feedback item at a time. Refer to the QA Feedback tab for each original requirement.</x:v>
+      </x:c>
+      <x:c r="E25" s="27" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="26"/>
+      <x:c r="B26" s="26"/>
+      <x:c r="C26" s="26"/>
+      <x:c r="D26" s="26"/>
+      <x:c r="E26" s="26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="26" t="str">
+        <x:v>Implementation commits</x:v>
+      </x:c>
+      <x:c r="B27" s="26"/>
+      <x:c r="C27" s="26" t="str">
+        <x:v>#1: 69e0d80d     #3: f6398f84</x:v>
+      </x:c>
+      <x:c r="D27" s="26"/>
+      <x:c r="E27" s="26"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="26" t="str">
+        <x:v>Verified code backup</x:v>
+      </x:c>
+      <x:c r="B28" s="26"/>
+      <x:c r="C28" s="26" t="str">
+        <x:v>Private jellygarden-codex repository, branch qa-feedback-20261007.</x:v>
+      </x:c>
+      <x:c r="D28" s="26"/>
+      <x:c r="E28" s="26"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="26"/>
+      <x:c r="B29" s="26"/>
+      <x:c r="C29" s="26"/>
+      <x:c r="D29" s="26"/>
+      <x:c r="E29" s="26"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="26" t="str">
+        <x:v>Evidence date</x:v>
+      </x:c>
+      <x:c r="B30" s="26"/>
+      <x:c r="C30" s="26" t="str">
+        <x:v>7 October 2026. Based on the recorded Unity checks and visual review.</x:v>
+      </x:c>
+      <x:c r="D30" s="26"/>
+      <x:c r="E30" s="26"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+    <x:mergeCell ref="A21:E21"/>
+    <x:mergeCell ref="A27:B27"/>
+    <x:mergeCell ref="C27:E27"/>
+    <x:mergeCell ref="A28:B28"/>
+    <x:mergeCell ref="C28:E28"/>
+    <x:mergeCell ref="A30:B30"/>
+    <x:mergeCell ref="C30:E30"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="E9:E19">
+    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Fixed"/>
+    <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Clarified"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb54ac70708546ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show one clear matching group for each hinted swap
</commit_message>
<xml_diff>
--- a/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
+++ b/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R9648dea607ec4963"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="Rd5d289435ac14867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R9b4004aaf9734bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="R08e2335e05bf4df1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -58,8 +58,14 @@
       <x:sz val="11"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF172554"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -94,6 +100,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -153,7 +164,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="63">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -294,11 +305,26 @@
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="8">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -373,6 +399,17 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -396,6 +433,19 @@
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="FixingReport" displayName="FixingReport" ref="A8:E19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Feedback"/>
+    <x:tableColumn id="2" name="Change"/>
+    <x:tableColumn id="3" name="Completed work"/>
+    <x:tableColumn id="4" name="Verification / evidence"/>
+    <x:tableColumn id="5" name="Tracker status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SingleMoveFixReport" displayName="SingleMoveFixReport" ref="A34:E38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Feedback"/>
     <x:tableColumn id="2" name="Change"/>
@@ -669,14 +719,14 @@
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Fixed")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
         <x:v>Open / pending</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Open")+COUNTIF(F9:F19,"In progress")</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
         <x:v>Clarified</x:v>
@@ -810,7 +860,7 @@
         <x:v>141 Unity checks passed, 0 failed, on 7 Oct 2026. Commit f6398f84. See Fixing Report for details. Phone QA pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="58" customHeight="1">
+    <x:row r="12" ht="72" customHeight="1">
       <x:c r="A12" s="28" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -821,17 +871,19 @@
         <x:v>The hint line can indicate multiple possible moves at the same time.</x:v>
       </x:c>
       <x:c r="D12" s="27" t="str">
-        <x:v>Show one clear legal swap at a time and identify only the two gems involved.</x:v>
+        <x:v>Outline one matching group for one legal swap. Keep the swap pair clear and preserve the approved glow and 1.0×–1.06× pulse in the marked area.</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
         <x:v>Hint / Logic</x:v>
       </x:c>
       <x:c r="F12" s="28" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="G12" s="28" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G12" s="28" t="str">
+        <x:v>✓</x:v>
+      </x:c>
       <x:c r="H12" s="27" t="str">
-        <x:v>Handle separately.</x:v>
+        <x:v>186 Unity checks passed, 0 failed, on 7 Oct 2026. Dual-result swaps and concurrent hints verified. See Fixing Report. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -1023,7 +1075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22236f5d483a4057"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1452cbffc24990"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1080,14 +1132,14 @@
       </x:c>
       <x:c r="B5" s="55" t="n">
         <x:f>'QA Feedback'!D5</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C5" s="47" t="str">
         <x:v>Open / pending</x:v>
       </x:c>
       <x:c r="D5" s="55" t="n">
         <x:f>'QA Feedback'!F5</x:f>
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E5" s="26"/>
     </x:row>
@@ -1355,7 +1407,7 @@
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="48" t="str">
-        <x:v>1, 3</x:v>
+        <x:v>1, 3, 4</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
         <x:v>Android and phone QA</x:v>
@@ -1364,28 +1416,18 @@
         <x:v>Desktop Unity verification is complete. No updated Android build or physical-phone run was performed.</x:v>
       </x:c>
       <x:c r="D23" s="27" t="str">
-        <x:v>Build the updated QA APK and review alignment, motion, glow and touch behaviour on physical phones.</x:v>
+        <x:v>Build the updated QA APK and review alignment, hint clarity, motion, glow and touch behaviour on physical phones.</x:v>
       </x:c>
       <x:c r="E23" s="27" t="str">
         <x:v>Pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="60" customHeight="1">
-      <x:c r="A24" s="48" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B24" s="27" t="str">
-        <x:v>Hint accuracy</x:v>
-      </x:c>
-      <x:c r="C24" s="27" t="str">
-        <x:v>The concern about the line indicating multiple moves remains a separate open QA item.</x:v>
-      </x:c>
-      <x:c r="D24" s="27" t="str">
-        <x:v>Investigate hint selection and the marked result before changing this behaviour.</x:v>
-      </x:c>
-      <x:c r="E24" s="27" t="str">
-        <x:v>Open</x:v>
-      </x:c>
+    <x:row r="24" ht="7" customHeight="1">
+      <x:c r="A24" s="48"/>
+      <x:c r="B24" s="27"/>
+      <x:c r="C24" s="27"/>
+      <x:c r="D24" s="27"/>
+      <x:c r="E24" s="27"/>
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="48" t="str">
@@ -1450,6 +1492,104 @@
       </x:c>
       <x:c r="D30" s="26"/>
       <x:c r="E30" s="26"/>
+    </x:row>
+    <x:row r="32" ht="27" customHeight="1">
+      <x:c r="A32" s="56" t="str">
+        <x:v>Feedback 4: one clear move suggestion</x:v>
+      </x:c>
+      <x:c r="B32" s="56"/>
+      <x:c r="C32" s="56"/>
+      <x:c r="D32" s="56"/>
+      <x:c r="E32" s="56"/>
+    </x:row>
+    <x:row r="34" ht="27" customHeight="1">
+      <x:c r="A34" s="61" t="str">
+        <x:v>Feedback</x:v>
+      </x:c>
+      <x:c r="B34" s="61" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="C34" s="61" t="str">
+        <x:v>Completed work</x:v>
+      </x:c>
+      <x:c r="D34" s="61" t="str">
+        <x:v>Verification / evidence</x:v>
+      </x:c>
+      <x:c r="E34" s="61" t="str">
+        <x:v>Tracker status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="70" customHeight="1">
+      <x:c r="A35" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B35" s="27" t="str">
+        <x:v>One marked match group</x:v>
+      </x:c>
+      <x:c r="C35" s="27" t="str">
+        <x:v>A swap that produces two coloured match groups now outlines only the strongest connected group. Both real match results remain available to gameplay.</x:v>
+      </x:c>
+      <x:c r="D35" s="27" t="str">
+        <x:v>Reproduced the original six-cell outline. Verified a single three-cell outline for the same swap after the fix.</x:v>
+      </x:c>
+      <x:c r="E35" s="48" t="str">
+        <x:f>'QA Feedback'!F12</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="70" customHeight="1">
+      <x:c r="A36" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B36" s="27" t="str">
+        <x:v>Stable choice and priority</x:v>
+      </x:c>
+      <x:c r="C36" s="27" t="str">
+        <x:v>Prioritizes the strongest matching pattern. Equal-result choices remain stable even when the swap partners are evaluated in reverse order.</x:v>
+      </x:c>
+      <x:c r="D36" s="27" t="str">
+        <x:v>Horizontal and vertical 3+3 and 3+4 cases, plus a 3+5 case, retain correct full match resolution and select one preview.</x:v>
+      </x:c>
+      <x:c r="E36" s="48" t="str">
+        <x:f>'QA Feedback'!F12</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="70" customHeight="1">
+      <x:c r="A37" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B37" s="27" t="str">
+        <x:v>One active hint</x:v>
+      </x:c>
+      <x:c r="C37" s="27" t="str">
+        <x:v>A new presenter retires the previous one. Multiple idle finders and alternative legal moves cannot accumulate additional suggestions.</x:v>
+      </x:c>
+      <x:c r="D37" s="27" t="str">
+        <x:v>Verified independent alternative swaps, three simultaneous idle finders, stable selection and presenter handoff.</x:v>
+      </x:c>
+      <x:c r="E37" s="48" t="str">
+        <x:f>'QA Feedback'!F12</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="70" customHeight="1">
+      <x:c r="A38" s="48" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B38" s="27" t="str">
+        <x:v>Existing interaction preserved</x:v>
+      </x:c>
+      <x:c r="C38" s="27" t="str">
+        <x:v>The marked group retains its brighter glow and 1.0×–1.06× pulse. Only the two swap partners move. Secondary result groups stay unmarked.</x:v>
+      </x:c>
+      <x:c r="D38" s="27" t="str">
+        <x:v>186 checks passed, 0 failed, in Unity 6000.5.10f1. Includes no-overlap, input, ownership and player-profile restoration checks.</x:v>
+      </x:c>
+      <x:c r="E38" s="48" t="str">
+        <x:f>'QA Feedback'!F12</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1462,14 +1602,19 @@
     <x:mergeCell ref="C28:E28"/>
     <x:mergeCell ref="A30:B30"/>
     <x:mergeCell ref="C30:E30"/>
+    <x:mergeCell ref="A32:E32"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E9:E19">
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Fixed"/>
     <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Clarified"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E35:E38">
+    <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Fixed"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb54ac70708546ba"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a54ec46b83849d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe7ee6e2227241d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rotate idle hints through other legal matching swaps
</commit_message>
<xml_diff>
--- a/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
+++ b/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R9b4004aaf9734bc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="R08e2335e05bf4df1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R94125a698b8f46cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="R8cd6fe01051e44cb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -405,7 +405,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -871,7 +871,7 @@
         <x:v>The hint line can indicate multiple possible moves at the same time.</x:v>
       </x:c>
       <x:c r="D12" s="27" t="str">
-        <x:v>Outline one matching group for one legal swap. Keep the swap pair clear and preserve the approved glow and 1.0×–1.06× pulse in the marked area.</x:v>
+        <x:v>Rotate through different legal swaps, one suggestion at a time. Show each for about 3.5 seconds before the next. Keep one marked group, the brighter glow and 1.0×–1.06× pulse.</x:v>
       </x:c>
       <x:c r="E12" s="26" t="str">
         <x:v>Hint / Logic</x:v>
@@ -883,7 +883,7 @@
         <x:v>✓</x:v>
       </x:c>
       <x:c r="H12" s="27" t="str">
-        <x:v>186 Unity checks passed, 0 failed, on 7 Oct 2026. Dual-result swaps and concurrent hints verified. See Fixing Report. Phone QA pending.</x:v>
+        <x:v>192 Unity checks passed, 0 failed, on 7 Oct 2026. Full rotation, unique choices, single marking, cleanup and cancellation verified. See Fixing Report. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="58" customHeight="1">
@@ -1075,7 +1075,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1452cbffc24990"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dcb44ff831641d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1542,13 +1542,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B36" s="27" t="str">
-        <x:v>Stable choice and priority</x:v>
+        <x:v>Different legal combinations</x:v>
       </x:c>
       <x:c r="C36" s="27" t="str">
-        <x:v>Prioritizes the strongest matching pattern. Equal-result choices remain stable even when the swap partners are evaluated in reverse order.</x:v>
+        <x:v>Starts with the strongest swap, then shows every other legal swap before repeating. Each remains visible for about 3.5 seconds, covering two interaction cycles.</x:v>
       </x:c>
       <x:c r="D36" s="27" t="str">
-        <x:v>Horizontal and vertical 3+3 and 3+4 cases, plus a 3+5 case, retain correct full match resolution and select one preview.</x:v>
+        <x:v>Verified all legal choices appear once per cycle, alternatives are shown, and the sequence wraps after all choices.</x:v>
       </x:c>
       <x:c r="E36" s="48" t="str">
         <x:f>'QA Feedback'!F12</x:f>
@@ -1563,10 +1563,10 @@
         <x:v>One active hint</x:v>
       </x:c>
       <x:c r="C37" s="27" t="str">
-        <x:v>A new presenter retires the previous one. Multiple idle finders and alternative legal moves cannot accumulate additional suggestions.</x:v>
+        <x:v>Only one suggestion is visible at a time. Switching clears the previous pose and glow. Input or board changes end the sequence and require a fresh idle delay.</x:v>
       </x:c>
       <x:c r="D37" s="27" t="str">
-        <x:v>Verified independent alternative swaps, three simultaneous idle finders, stable selection and presenter handoff.</x:v>
+        <x:v>Verified concurrent idle finders, presenter handoff, one outline throughout rotation, cleanup and immediate cancellation.</x:v>
       </x:c>
       <x:c r="E37" s="48" t="str">
         <x:f>'QA Feedback'!F12</x:f>
@@ -1584,7 +1584,7 @@
         <x:v>The marked group retains its brighter glow and 1.0×–1.06× pulse. Only the two swap partners move. Secondary result groups stay unmarked.</x:v>
       </x:c>
       <x:c r="D38" s="27" t="str">
-        <x:v>186 checks passed, 0 failed, in Unity 6000.5.10f1. Includes no-overlap, input, ownership and player-profile restoration checks.</x:v>
+        <x:v>192 checks passed, 0 failed, in Unity 6000.5.10f1. Includes rotation, no-overlap, input, ownership and player-profile restoration checks.</x:v>
       </x:c>
       <x:c r="E38" s="48" t="str">
         <x:f>'QA Feedback'!F12</x:f>
@@ -1613,8 +1613,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a54ec46b83849d9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe7ee6e2227241d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c502ca69e5542b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09cfe456bb1842bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix QA 5 super bomb fuse visibility and animated tip tracking
</commit_message>
<xml_diff>
--- a/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
+++ b/outputs/qa-feedback-tracker-20261007/Royal-Throne-QA-Feedback-Tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R94125a698b8f46cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="R8cd6fe01051e44cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA Feedback" sheetId="1" r:id="R989b86675cc94568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixing Report" sheetId="2" r:id="R31b42b5bb0184b56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -65,7 +65,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,6 +100,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEFF6FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1E3A8A"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -164,7 +169,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="63">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -320,11 +325,22 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="8">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -410,6 +426,17 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF166534"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFDCFCE7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
@@ -446,6 +473,19 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SingleMoveFixReport" displayName="SingleMoveFixReport" ref="A34:E38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
+    <x:tableColumn id="1" name="Feedback"/>
+    <x:tableColumn id="2" name="Change"/>
+    <x:tableColumn id="3" name="Completed work"/>
+    <x:tableColumn id="4" name="Verification / evidence"/>
+    <x:tableColumn id="5" name="Tracker status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SuperBombFuseFixReport" displayName="SuperBombFuseFixReport" ref="A42:E45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Feedback"/>
     <x:tableColumn id="2" name="Change"/>
@@ -719,14 +759,14 @@
       </x:c>
       <x:c r="D5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Fixed")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="10" t="str">
         <x:v>Open / pending</x:v>
       </x:c>
       <x:c r="F5" s="14" t="n">
         <x:f>COUNTIF(F9:F19,"Open")+COUNTIF(F9:F19,"In progress")</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G5" s="10" t="str">
         <x:v>Clarified</x:v>
@@ -886,7 +926,7 @@
         <x:v>192 Unity checks passed, 0 failed, on 7 Oct 2026. Full rotation, unique choices, single marking, cleanup and cancellation verified. See Fixing Report. Phone QA pending.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="58" customHeight="1">
+    <x:row r="13" ht="72" customHeight="1">
       <x:c r="A13" s="28" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -903,11 +943,13 @@
         <x:v>Animation / VFX</x:v>
       </x:c>
       <x:c r="F13" s="28" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="G13" s="28" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="G13" s="28" t="str">
+        <x:v>✓</x:v>
+      </x:c>
       <x:c r="H13" s="27" t="str">
-        <x:v>Handle separately.</x:v>
+        <x:v>22 Unity checks passed, 0 failed, on 7 Oct 2026. Visible fuse fire follows the rope at 30/60 FPS. See Fixing Report. Phone QA pending.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="58" customHeight="1">
@@ -1075,7 +1117,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dcb44ff831641d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R816b220310254a06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1132,14 +1174,14 @@
       </x:c>
       <x:c r="B5" s="55" t="n">
         <x:f>'QA Feedback'!D5</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="47" t="str">
         <x:v>Open / pending</x:v>
       </x:c>
       <x:c r="D5" s="55" t="n">
         <x:f>'QA Feedback'!F5</x:f>
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E5" s="26"/>
     </x:row>
@@ -1407,7 +1449,7 @@
     </x:row>
     <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="48" t="str">
-        <x:v>1, 3, 4</x:v>
+        <x:v>1, 3, 4, 5</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
         <x:v>Android and phone QA</x:v>
@@ -1416,7 +1458,7 @@
         <x:v>Desktop Unity verification is complete. No updated Android build or physical-phone run was performed.</x:v>
       </x:c>
       <x:c r="D23" s="27" t="str">
-        <x:v>Build the updated QA APK and review alignment, hint clarity, motion, glow and touch behaviour on physical phones.</x:v>
+        <x:v>Review alignment, hints, touch behaviour and super bomb fuse fire on physical phones with an updated QA APK.</x:v>
       </x:c>
       <x:c r="E23" s="27" t="str">
         <x:v>Pending</x:v>
@@ -1431,13 +1473,13 @@
     </x:row>
     <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="48" t="str">
-        <x:v>5–11</x:v>
+        <x:v>6–11</x:v>
       </x:c>
       <x:c r="B25" s="27" t="str">
         <x:v>Other original QA items</x:v>
       </x:c>
       <x:c r="C25" s="27" t="str">
-        <x:v>Fuse fire, special-piece creation, match timing, stuck gems, Color Ball duration and the 2×2-plus-one rule remain open.</x:v>
+        <x:v>Special-piece creation, match response, stuck/overlapping gems, Color Ball duration and square-plus-one Propeller detection remain open.</x:v>
       </x:c>
       <x:c r="D25" s="27" t="str">
         <x:v>Continue one feedback item at a time. Refer to the QA Feedback tab for each original requirement.</x:v>
@@ -1588,6 +1630,86 @@
       </x:c>
       <x:c r="E38" s="48" t="str">
         <x:f>'QA Feedback'!F12</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="27" customHeight="1">
+      <x:c r="A40" s="56" t="str">
+        <x:v>Feedback 5: visible fire on the super bomb fuse</x:v>
+      </x:c>
+      <x:c r="B40" s="56"/>
+      <x:c r="C40" s="56"/>
+      <x:c r="D40" s="56"/>
+      <x:c r="E40" s="56"/>
+    </x:row>
+    <x:row r="42" ht="27" customHeight="1">
+      <x:c r="A42" s="67" t="str">
+        <x:v>Feedback</x:v>
+      </x:c>
+      <x:c r="B42" s="67" t="str">
+        <x:v>Change</x:v>
+      </x:c>
+      <x:c r="C42" s="67" t="str">
+        <x:v>Completed work</x:v>
+      </x:c>
+      <x:c r="D42" s="67" t="str">
+        <x:v>Verification / evidence</x:v>
+      </x:c>
+      <x:c r="E42" s="67" t="str">
+        <x:v>Tracker status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="82" customHeight="1">
+      <x:c r="A43" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B43" s="27" t="str">
+        <x:v>Visible burning tip</x:v>
+      </x:c>
+      <x:c r="C43" s="27" t="str">
+        <x:v>The existing imported fire was emitting behind the super bomb. It now draws above the bomb body, revealing the bright burning tip and sparks.</x:v>
+      </x:c>
+      <x:c r="D43" s="27" t="str">
+        <x:v>Reproduced hidden fire before the fix; reviewed actual Unity captures before/after and through the burn.</x:v>
+      </x:c>
+      <x:c r="E43" s="48" t="str">
+        <x:f>'QA Feedback'!F13</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="82" customHeight="1">
+      <x:c r="A44" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B44" s="27" t="str">
+        <x:v>Follow the shrinking fuse</x:v>
+      </x:c>
+      <x:c r="C44" s="27" t="str">
+        <x:v>The fire follows the animated tip after animation updates, removing the one-frame position delay. Particle scale remains stable.</x:v>
+      </x:c>
+      <x:c r="D44" s="27" t="str">
+        <x:v>30 and 60 FPS: attached throughout 48 and 96 sampled burn frames. Pause/resume, explosion handoff, cleanup and pool reuse passed.</x:v>
+      </x:c>
+      <x:c r="E44" s="48" t="str">
+        <x:f>'QA Feedback'!F13</x:f>
+        <x:v>Fixed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="82" customHeight="1">
+      <x:c r="A45" s="48" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B45" s="27" t="str">
+        <x:v>Verification and scope</x:v>
+      </x:c>
+      <x:c r="C45" s="27" t="str">
+        <x:v>Two real bomb combinations completed. Original fuse animation, burn duration and explosion gameplay are retained. Player balance and lives restored.</x:v>
+      </x:c>
+      <x:c r="D45" s="27" t="str">
+        <x:v>22 checks passed, 0 failed, in Unity 6000.5.10f1; no Console errors. Evidence: Design/QaFeedback/05-SuperBombFuse. Physical-phone QA pending.</x:v>
+      </x:c>
+      <x:c r="E45" s="48" t="str">
+        <x:f>'QA Feedback'!F13</x:f>
         <x:v>Fixed</x:v>
       </x:c>
     </x:row>
@@ -1603,6 +1725,7 @@
     <x:mergeCell ref="A30:B30"/>
     <x:mergeCell ref="C30:E30"/>
     <x:mergeCell ref="A32:E32"/>
+    <x:mergeCell ref="A40:E40"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="E9:E19">
     <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Fixed"/>
@@ -1611,10 +1734,14 @@
   <x:conditionalFormatting sqref="E35:E38">
     <x:cfRule type="containsText" dxfId="7" priority="3" operator="containsText" text="Fixed"/>
   </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E43:E45">
+    <x:cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="Fixed"/>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c502ca69e5542b2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09cfe456bb1842bc"/>
+  <x:tableParts count="3">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red3a84353aa14e61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff12c5ad7a54567"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a303bb6d36d4d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>